<commit_message>
Update O2S clean-up list 25 Sep 2026.xlsx
</commit_message>
<xml_diff>
--- a/Claude outputs/O2S clean-up list 25 Sep 2026.xlsx
+++ b/Claude outputs/O2S clean-up list 25 Sep 2026.xlsx
@@ -666,7 +666,7 @@
     <row r="1">
       <c r="A1" s="5" t="inlineStr">
         <is>
-          <t>Supply Chain — Saad Jamal (with Zain Ghaffar)</t>
+          <t>Supply Chain — Saad Jamal · Warehouse: Muhammad Shoaib, Zain Ghaffar</t>
         </is>
       </c>
     </row>
@@ -967,17 +967,17 @@
       </c>
       <c r="E11" s="7" t="inlineStr">
         <is>
-          <t>About 15,792 packed and not yet shipped. DC 121 waits for the Plant Manager.</t>
+          <t>About 15,792 packed and not yet shipped. DC 121 is loading, with no gate pass yet.</t>
         </is>
       </c>
       <c r="F11" s="7" t="inlineStr">
         <is>
-          <t>Issue the gate pass for DC 121 once Fahim approves it.</t>
+          <t>Warehouse (Shoaib / Zain): issue the gate pass for DC 121. Saad: review it. Then Fahim approves.</t>
         </is>
       </c>
       <c r="G11" s="7" t="inlineStr">
         <is>
-          <t>Today → Gate Pass</t>
+          <t>Today → Gate Pass, then Review truck</t>
         </is>
       </c>
       <c r="H11" s="8" t="inlineStr"/>
@@ -1004,17 +1004,17 @@
       </c>
       <c r="E12" s="7" t="inlineStr">
         <is>
-          <t>8,000 packed not shipped. DC 120 waits for the Plant Manager.</t>
+          <t>8,000 packed not shipped. DC 120 is loading, with no gate pass yet.</t>
         </is>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>Issue the gate pass for DC 120 once Fahim approves it.</t>
+          <t>Warehouse (Shoaib / Zain): issue the gate pass for DC 120. Saad: review it. Then Fahim approves.</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
         <is>
-          <t>Today → Gate Pass</t>
+          <t>Today → Gate Pass, then Review truck</t>
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr"/>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="F13" s="7" t="inlineStr">
         <is>
-          <t>Confirm delivery of DC 118 with the date on the signed challan.</t>
+          <t>Whoever sent DC 118 confirms delivery with the date on the signed challan (from build 25e: the sender first, Saad after 1 day, Fahim after 2).</t>
         </is>
       </c>
       <c r="G13" s="7" t="inlineStr">
@@ -1786,17 +1786,17 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Delivery challan waiting for your approval.</t>
+          <t>Stuck since 23 Sep: the app sent you this job but refused you when you tapped it (fixed in build 25e).</t>
         </is>
       </c>
       <c r="F5" s="7" t="inlineStr">
         <is>
-          <t>Approve DC 120.</t>
+          <t>After the warehouse issues the gate pass and Saad reviews (or 2 hours pass), approve the DC and release the truck.</t>
         </is>
       </c>
       <c r="G5" s="7" t="inlineStr">
         <is>
-          <t>Today → Approve DC</t>
+          <t>Today → Approve DC and release truck</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr"/>
@@ -1823,17 +1823,17 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>Delivery challan waiting for your approval.</t>
+          <t>Same as DC 120.</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>Approve DC 121.</t>
+          <t>Same: after the gate pass and Saad’s review, approve and release.</t>
         </is>
       </c>
       <c r="G6" s="7" t="inlineStr">
         <is>
-          <t>Today → Approve DC</t>
+          <t>Today → Approve DC and release truck</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>

</xml_diff>